<commit_message>
Some analysis of sounds.dat and loading of sound effects
</commit_message>
<xml_diff>
--- a/File Research/cutscenes.xlsx
+++ b/File Research/cutscenes.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97E5F32-2D07-47EE-853A-FA6B6CD0F62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70F9513-D7FC-4337-9D7D-6D88AF7E0725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13425" xr2:uid="{2AD68F47-D934-4C71-AC61-3EC6CD4F6DA3}"/>
+    <workbookView xWindow="2438" yWindow="848" windowWidth="16680" windowHeight="11444" activeTab="2" xr2:uid="{2AD68F47-D934-4C71-AC61-3EC6CD4F6DA3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="functions" sheetId="1" r:id="rId1"/>
+    <sheet name="source" sheetId="2" r:id="rId2"/>
+    <sheet name="Cutscene flags" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="79">
   <si>
     <t>show-text</t>
   </si>
@@ -200,6 +201,75 @@
   </si>
   <si>
     <t>Plays Music theme given by arg[0]</t>
+  </si>
+  <si>
+    <t>Cleared in ending cutscene function</t>
+  </si>
+  <si>
+    <t>Cleared when setting up a pause</t>
+  </si>
+  <si>
+    <t>When set the pause function is ignored?</t>
+  </si>
+  <si>
+    <t>0x5B</t>
+  </si>
+  <si>
+    <t>Stores the pause duration in the pause function</t>
+  </si>
+  <si>
+    <t>0-7</t>
+  </si>
+  <si>
+    <t>0x3F</t>
+  </si>
+  <si>
+    <t>Stores the frame value in the pause function</t>
+  </si>
+  <si>
+    <t>0x3D</t>
+  </si>
+  <si>
+    <t>double check</t>
+  </si>
+  <si>
+    <t>Stores frame in (arg[0] in PlayToFrame)</t>
+  </si>
+  <si>
+    <t>0x3B</t>
+  </si>
+  <si>
+    <t>Possibly the number of linefeeds in the cutscene string. Set in function 1, cleared in function 2</t>
+  </si>
+  <si>
+    <t>0x39</t>
+  </si>
+  <si>
+    <t>Stores colour for cutscene subtitle (arg[0] in CutsceneDisplayString)</t>
+  </si>
+  <si>
+    <t>0x38</t>
+  </si>
+  <si>
+    <t>Possibly where the string is stored in memory??</t>
+  </si>
+  <si>
+    <t>0x22</t>
+  </si>
+  <si>
+    <t>Related to the string in a cutscene.</t>
+  </si>
+  <si>
+    <t>0x20</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>Bits</t>
+  </si>
+  <si>
+    <t>Offset</t>
   </si>
 </sst>
 </file>
@@ -241,9 +311,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -262,9 +335,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -302,7 +375,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -408,7 +481,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -550,7 +623,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1425,4 +1498,164 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F88B38-FB7A-42C7-BF8F-4A09B5B8947D}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="58.9296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B21">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>